<commit_message>
udpate generatoer and encv
</commit_message>
<xml_diff>
--- a/output/Deployment_Report.xlsx
+++ b/output/Deployment_Report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="47">
   <si>
     <t>Issue No.</t>
   </si>
@@ -22,131 +22,170 @@
     <t>Resolution</t>
   </si>
   <si>
-    <t>MSUG-SAIS-I004096</t>
-  </si>
-  <si>
-    <t>[SIS][ADMISSION LIST] Upon viewing admission details, "Year Applied" shows 2024 for newly applied student</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Root Cause:
-According on the code the Year applied is hardcoded
+    <t>WEBHOOK-I006066</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[LMS STUDENT][CLASS &gt; ATTENDANCE] Cannot time in if there are multiple schedules for the same day </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Root Cause:
+Schedule filtering used find() , which returned only the first matching schedule instead of all applicable schedules, resulting in inaccurate schedule validation and incorrectly disabling the Time In button.
+Resolution:
+Updated the schedule filtering to retrieve all applicable schedule records and validate the current time against the correct schedule, ensuring the Time In button is properly enabled.</t>
+  </si>
+  <si>
+    <t>WEBHOOK-I006029</t>
+  </si>
+  <si>
+    <t>[CAS] Error occurs even if no schedule conflict. Error -&gt; Conflict Room/Schedule</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Root Cause:
+Remove the validation in backend since its outdated
 Solution:
-Add mapping of where createdAt according to data where year is admitted
-Root Cause:
-According on the code the Year applied is hardcoded
+use the validation in frontend added by sir ariel and add validation for semesterId and academicYearId per schedule. Added column: ALTER TABLE public."SectionsSchedules" add column "academicYearId" int null ; ALTER TABLE public."SectionsSchedules" add column "semesterId" int null ;</t>
+  </si>
+  <si>
+    <t>WEBHOOK-I006013</t>
+  </si>
+  <si>
+    <t>[LMS STUDENT][CLASS &gt; ATTENDANCE] Students should only be allowed to time in on the current date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Root Cause:
+No existing validation to ensure that Time In is only enabled when the selected date is today.
 Solution:
-Add mapping of where createdAt according to data where year is admitted</t>
-  </si>
-  <si>
-    <t>MSUG-SAIS-I004302</t>
-  </si>
-  <si>
-    <t>[FIS][FACULTY] Initially displayed faculty load counts do not match the displayed counts  when clicking/viewing the faculty details</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Root Cause:
-The Receive data in the display is no other loads because he allow only teaching loads
+Added a validation to enable the Time In button only when the selected date is today.</t>
+  </si>
+  <si>
+    <t>WEBHOOK-I006020</t>
+  </si>
+  <si>
+    <t>[LMS STUDENT][CLASS] Incorrect displayed instructor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Root Cause:
+faculty_Fk can be passed directly through the payload, which may lead to data inconsistencies during student enrollment. The faculty assignment should have a single source of truth.
 Solution:
-Remove the filteration of removing the other loads</t>
-  </si>
-  <si>
-    <t>MSUG-SAIS-I003151</t>
-  </si>
-  <si>
-    <t>MSUG-SAIS-(Scholarship)</t>
-  </si>
-  <si>
-    <t>MR Link: Fix the issue on searching for students by creating a new api controller for enrollments and searching through include</t>
-  </si>
-  <si>
-    <t>MSUG-SAIS-I004026</t>
-  </si>
-  <si>
-    <t>[USER PORTAL] Displayed unit counts should be based on the credited units, not the number of rows/records</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Root Cause:
-The code was using data.value?.count ?? data?.count , which only counts records instead of summing the actual credit values from each row.
+Removed faculty_Fk from the payload and made it exclusively derived from section_Fk to maintain a single source of truth and prevent data inconsistencies. Added logic to retrieve the assigned instructor based on section_Fk . Note: updated document to remove faculty_Fk in student-enrolled payload</t>
+  </si>
+  <si>
+    <t>WEBHOOK-I006037</t>
+  </si>
+  <si>
+    <t>[CAS][SECTIONS] After deleting schedules through webhook, deleted schedules are still reflected when viewing the section schedules</t>
+  </si>
+  <si>
+    <t>fix is connected with this ticket:</t>
+  </si>
+  <si>
+    <t>WEBHOOK-I006025</t>
+  </si>
+  <si>
+    <t>[CAS][CAMPUS MANAGEMENT &gt; SECTION] Remove room assignment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Solution:
+remove room in code and uncomment codes for room that is unnecessary,</t>
+  </si>
+  <si>
+    <t>WEBHOOK-I006012</t>
+  </si>
+  <si>
+    <t>[LMS MOBILE][STUDENT] Inaccurate displayed schedule</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>WEBHOOK-I006119</t>
+  </si>
+  <si>
+    <t>[LMS STUDENT][EXCUSE REQUESTS] Only one schedule is displayed when a student has multiple shifts/schedules on the same day.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Root Cause:
+Section schedule data was not included in the LMS Section association, resulting in incomplete schedule information. Additionally, schedules under the same section and day were treated as duplicates.
+Resolution:
+Added the sectionSchedules association to the Section retrieval in LMS and updated the corresponding modals to map and display all associated schedules. Enhanced the filtering logic to consider the schedule time range, allowing multiple schedules under the same section and day to be displayed correctly.</t>
+  </si>
+  <si>
+    <t>WEBHOOK-I006115</t>
+  </si>
+  <si>
+    <t>[WEBHOOK][SCHEDULES] Type should only accept valid values</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Solution:
+add validation for type</t>
+  </si>
+  <si>
+    <t>WEBHOOK-I006069</t>
+  </si>
+  <si>
+    <t>[LMS INSTRUCTOR][EXCUSE REQUESTS] Only one schedule is displayed when a student has multiple shifts/schedules on the same day.</t>
+  </si>
+  <si>
+    <t>WEBHOOK-I006110</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[WEBHOOK][SCHEDULES] When deleting, isActive is set to False in the payload, but data remains active. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Root Cause:
+DELETE result was returning the old record instead of the updated record.
+Resolution:
+Return the updated record with isActive: false and deletedAt using findByIdAndUpdate() with { new: true } .</t>
+  </si>
+  <si>
+    <t>WEBHOOK-I006112</t>
+  </si>
+  <si>
+    <t>[WEBHOOK][SCHEDULES] Mode should only accept valid values</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Root Cause:
+no existing validation in code
 Solution:
-Replaced the count-based logic with reduce() to correctly compute the total credits by summing e.credit from data.rows .</t>
-  </si>
-  <si>
-    <t>MSUG-SAIS-I003149</t>
-  </si>
-  <si>
-    <t>SAIS - IAM - Uploading of Photo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">For Checking (PROD_ Network Issue in VM
-Fixed by SIr Josh STAGING June 8, 2026
-sync updating of avatar both in User and Employee Table</t>
-  </si>
-  <si>
-    <t>MSUG-SAIS-I004270</t>
-  </si>
-  <si>
-    <t>[ENROLLMENT - student] Upon clicking the notification bell, the notification box containing the notifications does not appear</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Screenshot 2026-06-10 at 10.05.33 AM.png current testing in local is working. Verify in dev live
-</t>
-  </si>
-  <si>
-    <t>MSUG-LMS-I004279</t>
-  </si>
-  <si>
-    <t>[LMS] Duplicating tab automatically logs out current session</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-Screenshot 2026-06-10 at 11.30.38 AM.png
-Passed (DEV) TEST RESULT: Issue still persists during testing. Upon duplicating the browser tab, the current session automatically expires and the user is logged out. The system displays a "Session Expired" message, indicating that the issue has not been resolved and requires further investigation.
-working as of current testing.
-This Nuxt plugin manages an SSE connection for real-time notifications (session-expiry warnings, OTP prompts, new notifications), reconnecting automatically when the tab is refocused. The fix adds an intentionallyDisconnected flag so a genuine server-side disconnect (e.g., session expiry) isn't silently undone by the tab-refocus reconnect logic, and replaces the unreliable onUnmounted cleanup with beforeunload .</t>
-  </si>
-  <si>
-    <t>MSUG-SAIS-I005158</t>
-  </si>
-  <si>
-    <t>[LMS INSTRUCTOR][QUESTIONNAIRE] Error 500 occurs when deleting and archiving/unarchiving a question (stg)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Root Cause:
-Missing null validation before accessing the length property caused the application to throw an error when the value was null. Screenshot 2026-07-20 at 1.47.55 PM.png
+added validation to display error and what values are only accepted. if(item.mode &amp;amp;&amp;amp; !["ONLINE", "FACE_TO_FACE"].includes(item.mode.toUpperCase())) {
+ throw {
+ message: `Invalid mode value [${item.mode}]. Allowed values are: FACE_TO_FACE and ONLINE only`,
+ status: 400,
+ };
+ }</t>
+  </si>
+  <si>
+    <t>WEBHOOK-I006107</t>
+  </si>
+  <si>
+    <t>[WEBHOOK] Creation of section still proceeded even if invalid room_Fk was supplied in the schedules</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Root Cause:
+Missing validation for invalid or non-existing room_Fk references in section schedules.
+Resolution:
+Added room reference validation to ensure that each provided room_Fk exists before processing the section schedule.</t>
+  </si>
+  <si>
+    <t>WEBHOOK-I006068</t>
+  </si>
+  <si>
+    <t>[WEBHOOK] Deletion should not succeed without section_fk</t>
+  </si>
+  <si>
+    <t>resolved by ticket:</t>
+  </si>
+  <si>
+    <t>WEBHOOK-I006022</t>
+  </si>
+  <si>
+    <t>[WEBHOOK][SECTION SCHEDULE] Missing section_Fk results in updating the schedule of another section</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Root Cause:
+no existing code for validating payload undefined values
 Solution:
-Added a null handler for length to prevent runtime errors.</t>
-  </si>
-  <si>
-    <t>MSUG-SAIS-I002936</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TRAINING NOTES [SIS] Student Assistant Module - Total duration (in hours) should be per month. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Root Cause:
-The duration is hours
-Solution:
-Make the duration from hours to months
-Root Cause:
-The total duration is hours instead of formatted duration of hours, minutes and seconds and wrong display
-Solution:
-The total duration is formatted by hours, minutes and seconds and it is depends on the data</t>
-  </si>
-  <si>
-    <t>MSUG-SAIS-I004091</t>
-  </si>
-  <si>
-    <t>[SIS][SCHOLARSHIPS] List of scholarship applications is not paginated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Root Cause:
-No pagination in the scholarship application
-Solution:
-Add pagination on this scholarship application only for gensan env
-Root Cause:
-No pagination in the scholarship application
-Solution:
-Add pagination on this scholarship application only for gensan env</t>
+added code for validating no undefined values for section_Fk</t>
   </si>
 </sst>
 </file>
@@ -523,7 +562,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -649,7 +688,62 @@
         <v>31</v>
       </c>
       <c r="C11" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>32</v>
+      </c>
+      <c r="B12" t="s">
+        <v>33</v>
+      </c>
+      <c r="C12" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>35</v>
+      </c>
+      <c r="B13" t="s">
+        <v>36</v>
+      </c>
+      <c r="C13" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>38</v>
+      </c>
+      <c r="B14" t="s">
+        <v>39</v>
+      </c>
+      <c r="C14" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>41</v>
+      </c>
+      <c r="B15" t="s">
+        <v>42</v>
+      </c>
+      <c r="C15" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>44</v>
+      </c>
+      <c r="B16" t="s">
+        <v>45</v>
+      </c>
+      <c r="C16" t="s">
+        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>